<commit_message>
Finalização do projeto ODS4
Finalizei o projeto escolar de PWEB do tema 4 das ODS's. Também adicionei o conteúdo das aulas que ainda não havia salvo
</commit_message>
<xml_diff>
--- a/PTIC/Maria Paula e Victor_ex19_ptic_Jorge Street.xlsx
+++ b/PTIC/Maria Paula e Victor_ex19_ptic_Jorge Street.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PTIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B3F59E2-FE79-4BD2-B919-B6FC50B10DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C529380-17FC-4D69-AC4D-11D940325C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1E232079-D0F3-4321-89F6-7B5D47D862B6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>Módulo/Área</t>
   </si>
@@ -107,9 +107,6 @@
     <t>alta</t>
   </si>
   <si>
-    <t>Área da Goleta</t>
-  </si>
-  <si>
     <t>Role a roleta para ganhar grana</t>
   </si>
   <si>
@@ -120,6 +117,39 @@
   </si>
   <si>
     <t>insirir as apostas do jogadores</t>
+  </si>
+  <si>
+    <t>Área da roleta</t>
+  </si>
+  <si>
+    <t>Área destinada para receber o dinheiro para apostar</t>
+  </si>
+  <si>
+    <t>Área do recebimento</t>
+  </si>
+  <si>
+    <t>O usuário receber o dinheiro das apostas</t>
+  </si>
+  <si>
+    <t>É a áreas destinada para os usuários receberem o dinheiro ganho nas suas apostas</t>
+  </si>
+  <si>
+    <t>Área do jogo da bomba</t>
+  </si>
+  <si>
+    <t>Acertar os lugares sem bomba para ganhar</t>
+  </si>
+  <si>
+    <t>Jogo para ganhar dinheiro caso o jogador acerte os quadrantes onde não tem a bomba, caso ele acerte, seu dinheiro aumente, do contrário, ele perderá tudo</t>
+  </si>
+  <si>
+    <t>Área da cartinha</t>
+  </si>
+  <si>
+    <t>Jogo estilo caça níqueis</t>
+  </si>
+  <si>
+    <t>Jogo onde  são sorteadas 3 cartas, caso elas sejam iguais, o dinheiro é multiplicado, a depender de qual carta foi acertada</t>
   </si>
 </sst>
 </file>
@@ -135,19 +165,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="5" tint="-0.499984740745262"/>
-      <name val="Century"/>
-      <family val="1"/>
-    </font>
-    <font>
       <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFC00000"/>
+      <name val="Century"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -159,7 +189,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor rgb="FFFE6666"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -193,23 +223,23 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -230,18 +260,13 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFE6666"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -251,6 +276,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>276225</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0E0A3A3-2B68-521B-FF47-5BEF3F050F64}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6562725" y="47625"/>
+          <a:ext cx="2409825" cy="2409825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -581,151 +661,171 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
+    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
+    <row r="9" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="B11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2" t="s">
+    <row r="12" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -734,11 +834,11 @@
     <mergeCell ref="A1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:E12">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Cancelado">
+      <formula>NOT(ISERROR(SEARCH("Cancelado",E5)))</formula>
+    </cfRule>
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Concluído">
       <formula>NOT(ISERROR(SEARCH("Concluído",E5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Cancelado">
-      <formula>NOT(ISERROR(SEARCH("Cancelado",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -747,5 +847,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>